<commit_message>
feat: enhance import script to auto-trigger checkin emails and skip completed guests
</commit_message>
<xml_diff>
--- a/reservations.xlsx
+++ b/reservations.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>First Name</t>
   </si>
@@ -73,10 +73,13 @@
     <t>Schmidt</t>
   </si>
   <si>
-    <t>laura.schmidt@example.com</t>
+    <t>molkamhissen@gmail.com</t>
   </si>
   <si>
     <t>Allemande</t>
+  </si>
+  <si>
+    <t>hotel-palais-bayram</t>
   </si>
   <si>
     <t>Marco</t>
@@ -536,7 +539,7 @@
         <v>46220.0</v>
       </c>
       <c r="G2" s="6">
-        <v>45127.0</v>
+        <v>46223.0</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>13</v>
@@ -562,7 +565,7 @@
         <v>46224.0</v>
       </c>
       <c r="G3" s="6">
-        <v>45121.0</v>
+        <v>46217.0</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>13</v>
@@ -585,30 +588,30 @@
         <v>21</v>
       </c>
       <c r="F4" s="6">
-        <v>46219.0</v>
+        <v>46220.0</v>
       </c>
       <c r="G4" s="6">
-        <v>45132.0</v>
+        <v>46228.0</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="5">
         <v>32405.0</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" s="6">
         <v>46226.0</v>
@@ -622,19 +625,19 @@
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="5">
         <v>34706.0</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" s="6">
         <v>46225.0</v>

</xml_diff>